<commit_message>
fix: add employee import migrations and templates
</commit_message>
<xml_diff>
--- a/public/templates/hr/employee_import_template.xlsx
+++ b/public/templates/hr/employee_import_template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rec30628f96d243c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees Import" sheetId="2" r:id="Rdfc56ed327094f55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Data" sheetId="3" r:id="R82a5997463214df8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup Lists" sheetId="4" r:id="R1240caf665c74ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example Row" sheetId="5" r:id="R3d490258448f42ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R97221a1169e74475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees Import" sheetId="2" r:id="Re1ea14244ccc454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Data" sheetId="3" r:id="Rf5336c15aed54cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup Lists" sheetId="4" r:id="Rab29b5beb2634413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example Row" sheetId="5" r:id="R3539945aeaa1431b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -232,7 +232,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="174">
+  <x:cellXfs count="175">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -641,6 +641,14 @@
     <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -918,7 +926,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="56" t="str">
-        <x:v>Use the Employees Import sheet to prepare employee records for the HR module. The workbook includes controlled dropdowns, date formats, payroll limits, and reference lists.</x:v>
+        <x:v>Use the Employees Import sheet to prepare employee records. Filament 3 imports CSV files, so complete the sheet, then save/export only the Employees Import sheet as CSV UTF-8 before uploading.</x:v>
       </x:c>
       <x:c r="B4" s="56"/>
       <x:c r="C4" s="56"/>
@@ -967,7 +975,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B8" s="60" t="str">
-        <x:v>Complete one employee per row in the Employees Import sheet. Do not rename or reorder the headers.</x:v>
+        <x:v>Replace or delete the three sample rows in Employees Import. Do not rename or reorder the headers.</x:v>
       </x:c>
       <x:c r="C8" s="54"/>
       <x:c r="D8" s="54"/>
@@ -981,7 +989,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B9" s="60" t="str">
-        <x:v>Required fields: first_name, last_name, id_passport_number, phone, and hire_date.</x:v>
+        <x:v>Department and Job Title values must already exist in the system and match exactly.</x:v>
       </x:c>
       <x:c r="C9" s="54"/>
       <x:c r="D9" s="54"/>
@@ -995,7 +1003,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B10" s="60" t="str">
-        <x:v>Department and job_title must match names already configured in the system. Update Reference Data first.</x:v>
+        <x:v>The manager column must contain an existing manager's employee number, or remain blank.</x:v>
       </x:c>
       <x:c r="C10" s="54"/>
       <x:c r="D10" s="54"/>
@@ -1009,7 +1017,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="60" t="str">
-        <x:v>Enter dates as YYYY-MM-DD, for example 2026-07-12.</x:v>
+        <x:v>Export the Employees Import sheet as CSV UTF-8. Upload the CSV, not the .xlsx workbook.</x:v>
       </x:c>
       <x:c r="C11" s="54"/>
       <x:c r="D11" s="54"/>
@@ -1384,10 +1392,10 @@
         <x:v>department</x:v>
       </x:c>
       <x:c r="V1" s="101" t="str">
-        <x:v>job_title</x:v>
+        <x:v>jobTitle</x:v>
       </x:c>
       <x:c r="W1" s="94" t="str">
-        <x:v>reporting_manager_employee_number</x:v>
+        <x:v>manager</x:v>
       </x:c>
       <x:c r="X1" s="101" t="str">
         <x:v>employment_type</x:v>
@@ -1472,160 +1480,406 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="133"/>
-      <x:c r="B2" s="134"/>
-      <x:c r="C2" s="134"/>
-      <x:c r="D2" s="134"/>
-      <x:c r="E2" s="133"/>
-      <x:c r="F2" s="133"/>
-      <x:c r="G2" s="133"/>
-      <x:c r="H2" s="133"/>
-      <x:c r="I2" s="133"/>
-      <x:c r="J2" s="133"/>
-      <x:c r="K2" s="134"/>
-      <x:c r="L2" s="134"/>
-      <x:c r="M2" s="134"/>
-      <x:c r="N2" s="135"/>
-      <x:c r="O2" s="134"/>
-      <x:c r="P2" s="134"/>
-      <x:c r="Q2" s="134"/>
-      <x:c r="R2" s="134"/>
-      <x:c r="S2" s="134"/>
-      <x:c r="T2" s="135"/>
-      <x:c r="U2" s="134"/>
-      <x:c r="V2" s="134"/>
-      <x:c r="W2" s="133"/>
-      <x:c r="X2" s="134"/>
-      <x:c r="Y2" s="134"/>
-      <x:c r="Z2" s="134"/>
-      <x:c r="AA2" s="135"/>
-      <x:c r="AB2" s="135"/>
-      <x:c r="AC2" s="136"/>
-      <x:c r="AD2" s="136"/>
-      <x:c r="AE2" s="136"/>
-      <x:c r="AF2" s="136"/>
-      <x:c r="AG2" s="134"/>
-      <x:c r="AH2" s="134"/>
-      <x:c r="AI2" s="134"/>
-      <x:c r="AJ2" s="133"/>
-      <x:c r="AK2" s="133"/>
-      <x:c r="AL2" s="133"/>
-      <x:c r="AM2" s="134"/>
-      <x:c r="AN2" s="134"/>
-      <x:c r="AO2" s="134"/>
-      <x:c r="AP2" s="134"/>
-      <x:c r="AQ2" s="134"/>
-      <x:c r="AR2" s="136"/>
-      <x:c r="AS2" s="136"/>
-      <x:c r="AT2" s="136"/>
-      <x:c r="AU2" s="136"/>
-      <x:c r="AV2" s="133"/>
-      <x:c r="AW2" s="135"/>
-      <x:c r="AX2" s="134"/>
+      <x:c r="A2" s="133" t="str"/>
+      <x:c r="B2" s="134" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="C2" s="134" t="str">
+        <x:v>Wanjiku</x:v>
+      </x:c>
+      <x:c r="D2" s="134" t="str">
+        <x:v>Kariuki</x:v>
+      </x:c>
+      <x:c r="E2" s="133" t="str">
+        <x:v>31000001</x:v>
+      </x:c>
+      <x:c r="F2" s="133" t="str">
+        <x:v>A010000001A</x:v>
+      </x:c>
+      <x:c r="G2" s="133" t="str">
+        <x:v>NSSF-DEMO-001</x:v>
+      </x:c>
+      <x:c r="H2" s="133" t="str">
+        <x:v>SHA-DEMO-001</x:v>
+      </x:c>
+      <x:c r="I2" s="133" t="str">
+        <x:v>0700000001</x:v>
+      </x:c>
+      <x:c r="J2" s="133" t="str"/>
+      <x:c r="K2" s="134" t="str">
+        <x:v>amina.kariuki@example.com</x:v>
+      </x:c>
+      <x:c r="L2" s="134" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="M2" s="134" t="str">
+        <x:v>Kenyan</x:v>
+      </x:c>
+      <x:c r="N2" s="135" t="n">
+        <x:v>34839</x:v>
+      </x:c>
+      <x:c r="O2" s="134" t="str">
+        <x:v>Nakuru</x:v>
+      </x:c>
+      <x:c r="P2" s="134" t="str">
+        <x:v>single</x:v>
+      </x:c>
+      <x:c r="Q2" s="134" t="str">
+        <x:v>Nakuru</x:v>
+      </x:c>
+      <x:c r="R2" s="134" t="str">
+        <x:v>Main Farm Staff Quarters</x:v>
+      </x:c>
+      <x:c r="S2" s="134" t="str">
+        <x:v>P.O. Box 100-20100</x:v>
+      </x:c>
+      <x:c r="T2" s="135" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="U2" s="134" t="str">
+        <x:v>Human Resource</x:v>
+      </x:c>
+      <x:c r="V2" s="134" t="str">
+        <x:v>HR Officer</x:v>
+      </x:c>
+      <x:c r="W2" s="133" t="str"/>
+      <x:c r="X2" s="134" t="str">
+        <x:v>permanent</x:v>
+      </x:c>
+      <x:c r="Y2" s="134" t="str">
+        <x:v>Main Farm</x:v>
+      </x:c>
+      <x:c r="Z2" s="134" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="AA2" s="135" t="str"/>
+      <x:c r="AB2" s="135" t="str"/>
+      <x:c r="AC2" s="136" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="AD2" s="136" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="AE2" s="136" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="AF2" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG2" s="134" t="str">
+        <x:v>bank</x:v>
+      </x:c>
+      <x:c r="AH2" s="134" t="str">
+        <x:v>KCB Bank</x:v>
+      </x:c>
+      <x:c r="AI2" s="134" t="str">
+        <x:v>Nakuru</x:v>
+      </x:c>
+      <x:c r="AJ2" s="133" t="str">
+        <x:v>1100000001</x:v>
+      </x:c>
+      <x:c r="AK2" s="133" t="str"/>
+      <x:c r="AL2" s="133" t="str"/>
+      <x:c r="AM2" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN2" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO2" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP2" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ2" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR2" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS2" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT2" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AU2" s="136" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="AV2" s="133" t="str"/>
+      <x:c r="AW2" s="135" t="str"/>
+      <x:c r="AX2" s="134" t="str">
+        <x:v>Sample record — replace before production import.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="133"/>
-      <x:c r="B3" s="134"/>
-      <x:c r="C3" s="134"/>
-      <x:c r="D3" s="134"/>
-      <x:c r="E3" s="133"/>
-      <x:c r="F3" s="133"/>
-      <x:c r="G3" s="133"/>
-      <x:c r="H3" s="133"/>
-      <x:c r="I3" s="133"/>
-      <x:c r="J3" s="133"/>
-      <x:c r="K3" s="134"/>
-      <x:c r="L3" s="134"/>
-      <x:c r="M3" s="134"/>
-      <x:c r="N3" s="135"/>
-      <x:c r="O3" s="134"/>
-      <x:c r="P3" s="134"/>
-      <x:c r="Q3" s="134"/>
-      <x:c r="R3" s="134"/>
-      <x:c r="S3" s="134"/>
-      <x:c r="T3" s="135"/>
-      <x:c r="U3" s="134"/>
-      <x:c r="V3" s="134"/>
-      <x:c r="W3" s="133"/>
-      <x:c r="X3" s="134"/>
-      <x:c r="Y3" s="134"/>
-      <x:c r="Z3" s="134"/>
-      <x:c r="AA3" s="135"/>
-      <x:c r="AB3" s="135"/>
-      <x:c r="AC3" s="136"/>
-      <x:c r="AD3" s="136"/>
-      <x:c r="AE3" s="136"/>
-      <x:c r="AF3" s="136"/>
-      <x:c r="AG3" s="134"/>
-      <x:c r="AH3" s="134"/>
-      <x:c r="AI3" s="134"/>
-      <x:c r="AJ3" s="133"/>
-      <x:c r="AK3" s="133"/>
-      <x:c r="AL3" s="133"/>
-      <x:c r="AM3" s="134"/>
-      <x:c r="AN3" s="134"/>
-      <x:c r="AO3" s="134"/>
-      <x:c r="AP3" s="134"/>
-      <x:c r="AQ3" s="134"/>
-      <x:c r="AR3" s="136"/>
-      <x:c r="AS3" s="136"/>
-      <x:c r="AT3" s="136"/>
-      <x:c r="AU3" s="136"/>
-      <x:c r="AV3" s="133"/>
-      <x:c r="AW3" s="135"/>
-      <x:c r="AX3" s="134"/>
+      <x:c r="A3" s="133" t="str"/>
+      <x:c r="B3" s="134" t="str">
+        <x:v>Brian</x:v>
+      </x:c>
+      <x:c r="C3" s="134" t="str">
+        <x:v>Kiptoo</x:v>
+      </x:c>
+      <x:c r="D3" s="134" t="str">
+        <x:v>Cheruiyot</x:v>
+      </x:c>
+      <x:c r="E3" s="133" t="str">
+        <x:v>31000002</x:v>
+      </x:c>
+      <x:c r="F3" s="133" t="str">
+        <x:v>A010000002B</x:v>
+      </x:c>
+      <x:c r="G3" s="133" t="str">
+        <x:v>NSSF-DEMO-002</x:v>
+      </x:c>
+      <x:c r="H3" s="133" t="str">
+        <x:v>SHA-DEMO-002</x:v>
+      </x:c>
+      <x:c r="I3" s="133" t="str">
+        <x:v>0700000002</x:v>
+      </x:c>
+      <x:c r="J3" s="133" t="str"/>
+      <x:c r="K3" s="134" t="str">
+        <x:v>brian.cheruiyot@example.com</x:v>
+      </x:c>
+      <x:c r="L3" s="134" t="str">
+        <x:v>male</x:v>
+      </x:c>
+      <x:c r="M3" s="134" t="str">
+        <x:v>Kenyan</x:v>
+      </x:c>
+      <x:c r="N3" s="135" t="n">
+        <x:v>33916</x:v>
+      </x:c>
+      <x:c r="O3" s="134" t="str">
+        <x:v>Baringo</x:v>
+      </x:c>
+      <x:c r="P3" s="134" t="str">
+        <x:v>married</x:v>
+      </x:c>
+      <x:c r="Q3" s="134" t="str">
+        <x:v>Baringo</x:v>
+      </x:c>
+      <x:c r="R3" s="134" t="str">
+        <x:v>Livestock Block 1</x:v>
+      </x:c>
+      <x:c r="S3" s="134" t="str">
+        <x:v>P.O. Box 200-30400</x:v>
+      </x:c>
+      <x:c r="T3" s="135" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="U3" s="134" t="str">
+        <x:v>Livestock</x:v>
+      </x:c>
+      <x:c r="V3" s="134" t="str">
+        <x:v>Livestock Attendant</x:v>
+      </x:c>
+      <x:c r="W3" s="133" t="str"/>
+      <x:c r="X3" s="134" t="str">
+        <x:v>contract</x:v>
+      </x:c>
+      <x:c r="Y3" s="134" t="str">
+        <x:v>Main Farm</x:v>
+      </x:c>
+      <x:c r="Z3" s="134" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="AA3" s="135" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="AB3" s="135" t="n">
+        <x:v>46569</x:v>
+      </x:c>
+      <x:c r="AC3" s="136" t="n">
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="AD3" s="136" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="AE3" s="136" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="AF3" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG3" s="134" t="str">
+        <x:v>mpesa</x:v>
+      </x:c>
+      <x:c r="AH3" s="134" t="str"/>
+      <x:c r="AI3" s="134" t="str"/>
+      <x:c r="AJ3" s="133" t="str"/>
+      <x:c r="AK3" s="133" t="str">
+        <x:v>0700000002</x:v>
+      </x:c>
+      <x:c r="AL3" s="133" t="str"/>
+      <x:c r="AM3" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN3" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO3" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP3" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ3" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR3" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS3" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT3" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AU3" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AV3" s="133" t="str"/>
+      <x:c r="AW3" s="135" t="str"/>
+      <x:c r="AX3" s="134" t="str">
+        <x:v>Sample contract employee.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="133"/>
-      <x:c r="B4" s="134"/>
-      <x:c r="C4" s="134"/>
-      <x:c r="D4" s="134"/>
-      <x:c r="E4" s="133"/>
-      <x:c r="F4" s="133"/>
-      <x:c r="G4" s="133"/>
-      <x:c r="H4" s="133"/>
-      <x:c r="I4" s="133"/>
-      <x:c r="J4" s="133"/>
-      <x:c r="K4" s="134"/>
-      <x:c r="L4" s="134"/>
-      <x:c r="M4" s="134"/>
-      <x:c r="N4" s="135"/>
-      <x:c r="O4" s="134"/>
-      <x:c r="P4" s="134"/>
-      <x:c r="Q4" s="134"/>
-      <x:c r="R4" s="134"/>
-      <x:c r="S4" s="134"/>
-      <x:c r="T4" s="135"/>
-      <x:c r="U4" s="134"/>
-      <x:c r="V4" s="134"/>
-      <x:c r="W4" s="133"/>
-      <x:c r="X4" s="134"/>
-      <x:c r="Y4" s="134"/>
-      <x:c r="Z4" s="134"/>
-      <x:c r="AA4" s="135"/>
-      <x:c r="AB4" s="135"/>
-      <x:c r="AC4" s="136"/>
-      <x:c r="AD4" s="136"/>
-      <x:c r="AE4" s="136"/>
-      <x:c r="AF4" s="136"/>
-      <x:c r="AG4" s="134"/>
-      <x:c r="AH4" s="134"/>
-      <x:c r="AI4" s="134"/>
-      <x:c r="AJ4" s="133"/>
-      <x:c r="AK4" s="133"/>
-      <x:c r="AL4" s="133"/>
-      <x:c r="AM4" s="134"/>
-      <x:c r="AN4" s="134"/>
-      <x:c r="AO4" s="134"/>
-      <x:c r="AP4" s="134"/>
-      <x:c r="AQ4" s="134"/>
-      <x:c r="AR4" s="136"/>
-      <x:c r="AS4" s="136"/>
-      <x:c r="AT4" s="136"/>
-      <x:c r="AU4" s="136"/>
-      <x:c r="AV4" s="133"/>
-      <x:c r="AW4" s="135"/>
-      <x:c r="AX4" s="134"/>
+      <x:c r="A4" s="133" t="str"/>
+      <x:c r="B4" s="134" t="str">
+        <x:v>Cynthia</x:v>
+      </x:c>
+      <x:c r="C4" s="134" t="str">
+        <x:v>Njeri</x:v>
+      </x:c>
+      <x:c r="D4" s="134" t="str">
+        <x:v>Mwangi</x:v>
+      </x:c>
+      <x:c r="E4" s="133" t="str">
+        <x:v>31000003</x:v>
+      </x:c>
+      <x:c r="F4" s="133" t="str">
+        <x:v>A010000003C</x:v>
+      </x:c>
+      <x:c r="G4" s="133" t="str">
+        <x:v>NSSF-DEMO-003</x:v>
+      </x:c>
+      <x:c r="H4" s="133" t="str">
+        <x:v>SHA-DEMO-003</x:v>
+      </x:c>
+      <x:c r="I4" s="133" t="str">
+        <x:v>0700000003</x:v>
+      </x:c>
+      <x:c r="J4" s="133" t="str"/>
+      <x:c r="K4" s="134" t="str">
+        <x:v>cynthia.mwangi@example.com</x:v>
+      </x:c>
+      <x:c r="L4" s="134" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="M4" s="134" t="str">
+        <x:v>Kenyan</x:v>
+      </x:c>
+      <x:c r="N4" s="135" t="n">
+        <x:v>35840</x:v>
+      </x:c>
+      <x:c r="O4" s="134" t="str">
+        <x:v>Nyeri</x:v>
+      </x:c>
+      <x:c r="P4" s="134" t="str">
+        <x:v>single</x:v>
+      </x:c>
+      <x:c r="Q4" s="134" t="str">
+        <x:v>Nakuru</x:v>
+      </x:c>
+      <x:c r="R4" s="134" t="str">
+        <x:v>Administration Office</x:v>
+      </x:c>
+      <x:c r="S4" s="134" t="str">
+        <x:v>P.O. Box 300-20100</x:v>
+      </x:c>
+      <x:c r="T4" s="135" t="n">
+        <x:v>46206</x:v>
+      </x:c>
+      <x:c r="U4" s="134" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="V4" s="134" t="str">
+        <x:v>Accountant</x:v>
+      </x:c>
+      <x:c r="W4" s="133" t="str"/>
+      <x:c r="X4" s="134" t="str">
+        <x:v>probation</x:v>
+      </x:c>
+      <x:c r="Y4" s="134" t="str">
+        <x:v>Head Office</x:v>
+      </x:c>
+      <x:c r="Z4" s="134" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="AA4" s="135" t="n">
+        <x:v>46206</x:v>
+      </x:c>
+      <x:c r="AB4" s="135" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="AC4" s="136" t="n">
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="AD4" s="136" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="AE4" s="136" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="AF4" s="136" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="AG4" s="134" t="str">
+        <x:v>airtel_money</x:v>
+      </x:c>
+      <x:c r="AH4" s="134" t="str"/>
+      <x:c r="AI4" s="134" t="str"/>
+      <x:c r="AJ4" s="133" t="str"/>
+      <x:c r="AK4" s="133" t="str"/>
+      <x:c r="AL4" s="133" t="str">
+        <x:v>0730000003</x:v>
+      </x:c>
+      <x:c r="AM4" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN4" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO4" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP4" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ4" s="174" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR4" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS4" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT4" s="136" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AU4" s="136" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="AV4" s="133" t="str"/>
+      <x:c r="AW4" s="135" t="str"/>
+      <x:c r="AX4" s="134" t="str">
+        <x:v>Sample probation employee.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="133"/>
@@ -14542,7 +14796,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaea24b5cbd74816"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R430511666f674892"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15096,10 +15350,10 @@
         <x:v>department</x:v>
       </x:c>
       <x:c r="V1" s="151" t="str">
-        <x:v>job_title</x:v>
+        <x:v>jobTitle</x:v>
       </x:c>
       <x:c r="W1" s="151" t="str">
-        <x:v>reporting_manager_employee_number</x:v>
+        <x:v>manager</x:v>
       </x:c>
       <x:c r="X1" s="151" t="str">
         <x:v>employment_type</x:v>
@@ -15195,10 +15449,10 @@
         <x:v>Kariuki</x:v>
       </x:c>
       <x:c r="E2" s="161" t="str">
-        <x:v>00000000</x:v>
+        <x:v>31000001</x:v>
       </x:c>
       <x:c r="F2" s="161" t="str">
-        <x:v>A000000000A</x:v>
+        <x:v>A010000001A</x:v>
       </x:c>
       <x:c r="G2" s="161" t="str">
         <x:v>NSSF-DEMO-001</x:v>
@@ -15207,11 +15461,11 @@
         <x:v>SHA-DEMO-001</x:v>
       </x:c>
       <x:c r="I2" s="161" t="str">
-        <x:v>0700000000</x:v>
+        <x:v>0700000001</x:v>
       </x:c>
       <x:c r="J2" s="161" t="str"/>
       <x:c r="K2" s="157" t="str">
-        <x:v>amina.example@example.com</x:v>
+        <x:v>amina.kariuki@example.com</x:v>
       </x:c>
       <x:c r="L2" s="157" t="str">
         <x:v>female</x:v>
@@ -15219,8 +15473,8 @@
       <x:c r="M2" s="157" t="str">
         <x:v>Kenyan</x:v>
       </x:c>
-      <x:c r="N2" s="163" t="str">
-        <x:v>1995-05-20</x:v>
+      <x:c r="N2" s="163" t="n">
+        <x:v>34839</x:v>
       </x:c>
       <x:c r="O2" s="157" t="str">
         <x:v>Nakuru</x:v>
@@ -15232,13 +15486,13 @@
         <x:v>Nakuru</x:v>
       </x:c>
       <x:c r="R2" s="157" t="str">
-        <x:v>Example address</x:v>
+        <x:v>Main Farm Staff Quarters</x:v>
       </x:c>
       <x:c r="S2" s="157" t="str">
-        <x:v>P.O. Box 0000-00000</x:v>
-      </x:c>
-      <x:c r="T2" s="163" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>P.O. Box 100-20100</x:v>
+      </x:c>
+      <x:c r="T2" s="163" t="n">
+        <x:v>46204</x:v>
       </x:c>
       <x:c r="U2" s="157" t="str">
         <x:v>Human Resource</x:v>
@@ -15280,7 +15534,7 @@
         <x:v>Nakuru</x:v>
       </x:c>
       <x:c r="AJ2" s="161" t="str">
-        <x:v>0000000000</x:v>
+        <x:v>1100000001</x:v>
       </x:c>
       <x:c r="AK2" s="161" t="str"/>
       <x:c r="AL2" s="161" t="str"/>
@@ -15309,12 +15563,280 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="AU2" s="165" t="n">
-        <x:v>0</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="AV2" s="161" t="str"/>
       <x:c r="AW2" s="163" t="str"/>
       <x:c r="AX2" s="157" t="str">
-        <x:v>Fictional example only. Delete before use.</x:v>
+        <x:v>Sample record — replace before production import.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str"/>
+      <x:c r="B3" t="str">
+        <x:v>Brian</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Kiptoo</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Cheruiyot</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>31000002</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>A010000002B</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>NSSF-DEMO-002</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>SHA-DEMO-002</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>0700000002</x:v>
+      </x:c>
+      <x:c r="J3" t="str"/>
+      <x:c r="K3" t="str">
+        <x:v>brian.cheruiyot@example.com</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>male</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>Kenyan</x:v>
+      </x:c>
+      <x:c r="N3" s="105" t="n">
+        <x:v>33916</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>Baringo</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>married</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>Baringo</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:v>Livestock Block 1</x:v>
+      </x:c>
+      <x:c r="S3" t="str">
+        <x:v>P.O. Box 200-30400</x:v>
+      </x:c>
+      <x:c r="T3" s="105" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="U3" t="str">
+        <x:v>Livestock</x:v>
+      </x:c>
+      <x:c r="V3" t="str">
+        <x:v>Livestock Attendant</x:v>
+      </x:c>
+      <x:c r="W3" t="str"/>
+      <x:c r="X3" t="str">
+        <x:v>contract</x:v>
+      </x:c>
+      <x:c r="Y3" t="str">
+        <x:v>Main Farm</x:v>
+      </x:c>
+      <x:c r="Z3" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="AA3" s="105" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="AB3" s="105" t="n">
+        <x:v>46569</x:v>
+      </x:c>
+      <x:c r="AC3" t="n">
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="AD3" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="AE3" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="AF3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG3" t="str">
+        <x:v>mpesa</x:v>
+      </x:c>
+      <x:c r="AH3" t="str"/>
+      <x:c r="AI3" t="str"/>
+      <x:c r="AJ3" t="str"/>
+      <x:c r="AK3" t="str">
+        <x:v>0700000002</x:v>
+      </x:c>
+      <x:c r="AL3" t="str"/>
+      <x:c r="AM3" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN3" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO3" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP3" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ3" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AU3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AV3" t="str"/>
+      <x:c r="AW3" s="105" t="str"/>
+      <x:c r="AX3" t="str">
+        <x:v>Sample contract employee.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str"/>
+      <x:c r="B4" t="str">
+        <x:v>Cynthia</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Njeri</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Mwangi</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>31000003</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>A010000003C</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>NSSF-DEMO-003</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>SHA-DEMO-003</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>0700000003</x:v>
+      </x:c>
+      <x:c r="J4" t="str"/>
+      <x:c r="K4" t="str">
+        <x:v>cynthia.mwangi@example.com</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Kenyan</x:v>
+      </x:c>
+      <x:c r="N4" s="105" t="n">
+        <x:v>35840</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>Nyeri</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>single</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>Nakuru</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
+        <x:v>Administration Office</x:v>
+      </x:c>
+      <x:c r="S4" t="str">
+        <x:v>P.O. Box 300-20100</x:v>
+      </x:c>
+      <x:c r="T4" s="105" t="n">
+        <x:v>46206</x:v>
+      </x:c>
+      <x:c r="U4" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="V4" t="str">
+        <x:v>Accountant</x:v>
+      </x:c>
+      <x:c r="W4" t="str"/>
+      <x:c r="X4" t="str">
+        <x:v>probation</x:v>
+      </x:c>
+      <x:c r="Y4" t="str">
+        <x:v>Head Office</x:v>
+      </x:c>
+      <x:c r="Z4" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="AA4" s="105" t="n">
+        <x:v>46206</x:v>
+      </x:c>
+      <x:c r="AB4" s="105" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="AC4" t="n">
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="AD4" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="AE4" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="AF4" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="AG4" t="str">
+        <x:v>airtel_money</x:v>
+      </x:c>
+      <x:c r="AH4" t="str"/>
+      <x:c r="AI4" t="str"/>
+      <x:c r="AJ4" t="str"/>
+      <x:c r="AK4" t="str"/>
+      <x:c r="AL4" t="str">
+        <x:v>0730000003</x:v>
+      </x:c>
+      <x:c r="AM4" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN4" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO4" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP4" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ4" s="152" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AU4" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="AV4" t="str"/>
+      <x:c r="AW4" s="105" t="str"/>
+      <x:c r="AX4" t="str">
+        <x:v>Sample probation employee.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>